<commit_message>
release: iSurvey 1.4.0 — one bundle for AutoCAD and Civil 3D 2023-2027.
Each year loads the DLL built for its .NET runtime, so 2023 through 2027 are not forced onto a single binary.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AIProject\isurvey\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{517D7EC6-59CF-45EA-8661-64650842449C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D0CC6A-8855-4780-B962-05259FB14CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh sach lenh" sheetId="1" r:id="rId1"/>
     <sheet name="Mau chuan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="116">
   <si>
     <t>STT</t>
   </si>
@@ -253,6 +253,144 @@
   </si>
   <si>
     <t>ISURVEY_* luôn là lệnh chính; Shortcut chỉ là alias — đụng thì đổi alias, không đổi tên dài.</t>
+  </si>
+  <si>
+    <t>Khung &amp; Cắt Bình Đồ</t>
+  </si>
+  <si>
+    <t>Cắt Bình Đồ</t>
+  </si>
+  <si>
+    <t>CATBD</t>
+  </si>
+  <si>
+    <t>CBD</t>
+  </si>
+  <si>
+    <t>Cắt Bình Đồ — cắt theo biên khép kín</t>
+  </si>
+  <si>
+    <t>Cắt đối tượng theo đường biên khép kín: giữ Z, nội suy đoạn cắt, bảo vệ layer khung. Không dùng TRIM; UNDO một lần. Cần đã kích hoạt.</t>
+  </si>
+  <si>
+    <t>Model Space → CBD hoặc CATBD → chọn polyline khép kín → quét chọn bản vẽ (gõ ALL để chọn hết).</t>
+  </si>
+  <si>
+    <t>1.2.0</t>
+  </si>
+  <si>
+    <t>Hồ sơ &amp; QA/QC</t>
+  </si>
+  <si>
+    <t>Quét Cấu Trúc (AutoScan)</t>
+  </si>
+  <si>
+    <t>AUTOSCAN</t>
+  </si>
+  <si>
+    <t>SCN</t>
+  </si>
+  <si>
+    <t>Scan — quét cấu trúc (không dùng ASC: Telex thành "ác")</t>
+  </si>
+  <si>
+    <t>Quét vùng chọn, xuất CAD_AutoScan_Report.txt (thống kê nhóm, mẫu chữ, mẫu đại diện) rồi mở Notepad. Cần đã kích hoạt.</t>
+  </si>
+  <si>
+    <t>SCN hoặc AUTOSCAN → quét chọn khu vực (gõ ALL để chọn hết) → lưu file .txt.</t>
+  </si>
+  <si>
+    <t>Tài khoản &amp; Hệ thống</t>
+  </si>
+  <si>
+    <t>Đăng Nhập / Kích Hoạt</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGIN</t>
+  </si>
+  <si>
+    <t>LGI</t>
+  </si>
+  <si>
+    <t>Login — đăng nhập / kích hoạt Gmail</t>
+  </si>
+  <si>
+    <t>Gmail + OTP 6 số, tự xác thực khi đủ số. Tối đa 2 thiết bị. Panel 1–5 khóa khi chưa kích hoạt. Lệnh này không bị khóa.</t>
+  </si>
+  <si>
+    <t>LGI hoặc nút Ribbon → nhập Gmail → Gửi mã → nhập 6 số. Đã kích hoạt thì mở thông tin tài khoản.</t>
+  </si>
+  <si>
+    <t>1.3.0</t>
+  </si>
+  <si>
+    <t>Kiểm Tra Cập Nhật</t>
+  </si>
+  <si>
+    <t>ISURVEY_UPDATE</t>
+  </si>
+  <si>
+    <t>UPD</t>
+  </si>
+  <si>
+    <t>Update — kiểm tra phiên bản</t>
+  </si>
+  <si>
+    <t>Hiện phiên bản đang dùng. Chưa tự kiểm tra bản mới trên mạng. Không bị khóa khi chưa đăng nhập.</t>
+  </si>
+  <si>
+    <t>UPD hoặc nút Kiểm Tra Cập Nhật trên Ribbon.</t>
+  </si>
+  <si>
+    <t>Thông Tin &amp; Giấy Phép</t>
+  </si>
+  <si>
+    <t>ISURVEY_ABOUT</t>
+  </si>
+  <si>
+    <t>ABT</t>
+  </si>
+  <si>
+    <t>About — thông tin giấy phép</t>
+  </si>
+  <si>
+    <t>Hiện phiên bản, Gmail, mã thiết bị, ngày kích hoạt và hạn dùng khi mất mạng.</t>
+  </si>
+  <si>
+    <t>ABT hoặc nút Thông Tin &amp; Giấy Phép. Đã đăng nhập thì LGI cũng mở cửa sổ này.</t>
+  </si>
+  <si>
+    <t>Đăng Xuất / Đổi Máy</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGOUT</t>
+  </si>
+  <si>
+    <t>LGO</t>
+  </si>
+  <si>
+    <t>Logout — đăng xuất, trả suất thiết bị</t>
+  </si>
+  <si>
+    <t>Xóa giấy phép trên máy này và khóa panel 1–5. Nếu đang trực tuyến, trả suất để kích hoạt máy khác.</t>
+  </si>
+  <si>
+    <t>LGO hoặc nút Đăng Xuất / Đổi Máy → xác nhận. Nút Ribbon chỉ bật khi đã đăng nhập.</t>
+  </si>
+  <si>
+    <t>(Admin) Sinh mã OTP</t>
+  </si>
+  <si>
+    <t>ISURVEY_GENOTP</t>
+  </si>
+  <si>
+    <t>Không có alias — chỉ máy Admin</t>
+  </si>
+  <si>
+    <t>In mã 6 số trong ngày cho một Gmail. Chỉ chạy khi máy có AdminSecret trong auth.config.json. Không có nút Ribbon.</t>
+  </si>
+  <si>
+    <t>Máy Admin: gõ ISURVEY_GENOTP → nhập Gmail người dùng.</t>
   </si>
 </sst>
 </file>
@@ -708,22 +846,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}">
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.59765625" customWidth="1"/>
-    <col min="2" max="2" width="12.59765625" customWidth="1"/>
-    <col min="3" max="3" width="24.59765625" customWidth="1"/>
-    <col min="4" max="4" width="22.59765625" customWidth="1"/>
-    <col min="5" max="5" width="10.59765625" customWidth="1"/>
-    <col min="6" max="6" width="36.59765625" customWidth="1"/>
-    <col min="7" max="8" width="48.59765625" customWidth="1"/>
-    <col min="9" max="9" width="10.59765625" customWidth="1"/>
-    <col min="10" max="10" width="14.59765625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="28.59765625" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="2" max="2" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="24.5546875" customWidth="1"/>
+    <col min="4" max="4" width="22.5546875" customWidth="1"/>
+    <col min="5" max="5" width="10.5546875" customWidth="1"/>
+    <col min="6" max="6" width="36.5546875" customWidth="1"/>
+    <col min="7" max="8" width="48.5546875" customWidth="1"/>
+    <col min="9" max="9" width="10.5546875" customWidth="1"/>
+    <col min="10" max="10" width="14.5546875" style="6" customWidth="1"/>
+    <col min="11" max="11" width="28.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -758,7 +896,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -793,7 +931,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -828,7 +966,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -863,7 +1001,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -898,7 +1036,251 @@
         <v>30</v>
       </c>
     </row>
+    <row r="6" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="J6" s="3">
+        <v>46307</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="4">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" s="5">
+        <v>46307</v>
+      </c>
+      <c r="K7" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J8" s="3">
+        <v>46307</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J9" s="5">
+        <v>46307</v>
+      </c>
+      <c r="K9" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" s="3">
+        <v>46307</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="5">
+        <v>46307</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J12" s="3">
+        <v>46307</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:K12" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -906,13 +1288,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B0ECC91-F81E-481F-BB81-DBB8A841A6BC}">
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.59765625" customWidth="1"/>
-    <col min="2" max="2" width="70.59765625" customWidth="1"/>
+    <col min="1" max="1" width="36.5546875" customWidth="1"/>
+    <col min="2" max="2" width="70.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
@@ -920,12 +1302,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -933,7 +1315,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -941,7 +1323,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -949,7 +1331,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -957,7 +1339,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -965,7 +1347,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -973,7 +1355,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -981,12 +1363,12 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -994,7 +1376,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -1002,7 +1384,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1010,12 +1392,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
@@ -1023,7 +1405,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>2</v>
       </c>
@@ -1031,7 +1413,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>3</v>
       </c>
@@ -1039,7 +1421,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>4</v>
       </c>
@@ -1047,7 +1429,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>5</v>
       </c>
@@ -1055,7 +1437,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -1063,12 +1445,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="11" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>62</v>
       </c>
@@ -1076,7 +1458,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -1084,7 +1466,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>66</v>
       </c>
@@ -1092,7 +1474,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>68</v>
       </c>

</xml_diff>

<commit_message>
Phat hanh 1.8.10: nhap va xuat diem do, STT tren layer iSurvey_STT.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49D0CC6A-8855-4780-B962-05259FB14CE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB198ACD-DB81-4879-BFC7-B44DEC77AD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh sach lenh" sheetId="1" r:id="rId1"/>
     <sheet name="Mau chuan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="341">
   <si>
     <t>STT</t>
   </si>
@@ -135,9 +135,6 @@
     <t>1.1.0</t>
   </si>
   <si>
-    <t>Hoàn thành (cần cài bundle lại)</t>
-  </si>
-  <si>
     <t>Cột / Mục</t>
   </si>
   <si>
@@ -207,9 +204,6 @@
     <t>XG</t>
   </si>
   <si>
-    <t>EG</t>
-  </si>
-  <si>
     <t>Ý nghĩa (nghĩa nhớ)</t>
   </si>
   <si>
@@ -222,9 +216,6 @@
     <t>Xóa Google — xóa tile GE</t>
   </si>
   <si>
-    <t>Export Google — xuất KML/KMZ</t>
-  </si>
-  <si>
     <t>Giải thích mnemonic của Shortcut; đặt ngay sau cột Shortcut</t>
   </si>
   <si>
@@ -336,12 +327,6 @@
     <t>Update — kiểm tra phiên bản</t>
   </si>
   <si>
-    <t>Hiện phiên bản đang dùng. Chưa tự kiểm tra bản mới trên mạng. Không bị khóa khi chưa đăng nhập.</t>
-  </si>
-  <si>
-    <t>UPD hoặc nút Kiểm Tra Cập Nhật trên Ribbon.</t>
-  </si>
-  <si>
     <t>Thông Tin &amp; Giấy Phép</t>
   </si>
   <si>
@@ -391,6 +376,696 @@
   </si>
   <si>
     <t>Máy Admin: gõ ISURVEY_GENOTP → nhập Gmail người dùng.</t>
+  </si>
+  <si>
+    <t>EG, EXK</t>
+  </si>
+  <si>
+    <t>Export Google / Export KML — xuất KML/KMZ</t>
+  </si>
+  <si>
+    <t>Kiểm tra bản mới. Có bản thì tải và cài sau khi thoát Civil.</t>
+  </si>
+  <si>
+    <t>UPD hoặc nút Kiểm Tra Cập Nhật → Cập nhật ngay / Đóng.</t>
+  </si>
+  <si>
+    <t>1.8.6</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>Nhập File KML/KMZ</t>
+  </si>
+  <si>
+    <t>ISURVEY_IMPORT_KML</t>
+  </si>
+  <si>
+    <t>INK</t>
+  </si>
+  <si>
+    <t>Import KML — nhập KML/KMZ</t>
+  </si>
+  <si>
+    <t>Nhập KML/KMZ về tọa độ VN-2000 theo kinh tuyến đã chọn.</t>
+  </si>
+  <si>
+    <t>INK hoặc nút Nhập File KML/KMZ → chọn file.</t>
+  </si>
+  <si>
+    <t>1.5.0</t>
+  </si>
+  <si>
+    <t>13/10/2026</t>
+  </si>
+  <si>
+    <t>Cập Nhật Ảnh GE</t>
+  </si>
+  <si>
+    <t>ISURVEY_UPDATE_GE</t>
+  </si>
+  <si>
+    <t>Tải lại tile Google Earth theo khung nhìn hiện tại.</t>
+  </si>
+  <si>
+    <t>Model Space → nút Cập Nhật Ảnh GE. Cần đã chèn ảnh trước.</t>
+  </si>
+  <si>
+    <t>Nhập TAB → CAD</t>
+  </si>
+  <si>
+    <t>ISURVEY_TAB_TO_CAD</t>
+  </si>
+  <si>
+    <t>T2C</t>
+  </si>
+  <si>
+    <t>TAB to CAD — nhập MapInfo</t>
+  </si>
+  <si>
+    <t>Nhập TAB: tô màu MapInfo, layer theo MDSD, nhãn trong thửa. Đổi TM khi kinh tuyến khác bản vẽ.</t>
+  </si>
+  <si>
+    <t>T2C → chọn file TAB.</t>
+  </si>
+  <si>
+    <t>1.8.1</t>
+  </si>
+  <si>
+    <t>22/10/2026</t>
+  </si>
+  <si>
+    <t>Nhập DGN → CAD</t>
+  </si>
+  <si>
+    <t>ISURVEY_DGN_TO_CAD</t>
+  </si>
+  <si>
+    <t>D2C</t>
+  </si>
+  <si>
+    <t>DGN to CAD</t>
+  </si>
+  <si>
+    <t>Nhập DGN V7/V8 vào bản vẽ hiện hành, hoặc chuyển nhiều file sang DWG.</t>
+  </si>
+  <si>
+    <t>D2C → chọn file, ghép hoặc tách.</t>
+  </si>
+  <si>
+    <t>1.6.0</t>
+  </si>
+  <si>
+    <t>15/10/2026</t>
+  </si>
+  <si>
+    <t>Xuất CAD → DGN</t>
+  </si>
+  <si>
+    <t>ISURVEY_CAD_TO_DGN</t>
+  </si>
+  <si>
+    <t>C2D</t>
+  </si>
+  <si>
+    <t>CAD to DGN</t>
+  </si>
+  <si>
+    <t>Xuất DWG sang DGN V7 hoặc V8, seed VN-2000.</t>
+  </si>
+  <si>
+    <t>C2D → chọn phạm vi, phiên bản → lưu file.</t>
+  </si>
+  <si>
+    <t>Cấu Hình DGN</t>
+  </si>
+  <si>
+    <t>ISURVEY_DGN_CONFIG</t>
+  </si>
+  <si>
+    <t>DGNCFG</t>
+  </si>
+  <si>
+    <t>DGN config — đơn vị, layer, font</t>
+  </si>
+  <si>
+    <t>Lưu đơn vị, ánh xạ level sang layer, font TCVN3 sang Unicode.</t>
+  </si>
+  <si>
+    <t>DGNCFG → sửa bảng ánh xạ.</t>
+  </si>
+  <si>
+    <t>UAV &amp; LiDAR</t>
+  </si>
+  <si>
+    <t>Cắt Ảnh Theo Biên</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_CLIP</t>
+  </si>
+  <si>
+    <t>UAVCLIP</t>
+  </si>
+  <si>
+    <t>UAV clip — cắt ảnh theo biên</t>
+  </si>
+  <si>
+    <t>Cắt ảnh UAV theo polyline kín, hoặc tự cắt nền trắng-đen.</t>
+  </si>
+  <si>
+    <t>UAVCLIP → chọn ảnh → 1 polyline / 2 nền trắng-đen.</t>
+  </si>
+  <si>
+    <t>1.7.0</t>
+  </si>
+  <si>
+    <t>19/10/2026</t>
+  </si>
+  <si>
+    <t>Tắt/Bật Khung Ảnh</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_FRAME_TOGGLE</t>
+  </si>
+  <si>
+    <t>Bật hoặc tắt khung bao quanh ảnh raster.</t>
+  </si>
+  <si>
+    <t>Nút Tắt/Bật Khung Ảnh, hoặc gõ ISURVEY_UAV_FRAME_TOGGLE.</t>
+  </si>
+  <si>
+    <t>Đưa Ảnh Xuống Dưới</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_SEND_BACK</t>
+  </si>
+  <si>
+    <t>Đưa ảnh raster xuống dưới cùng thứ tự vẽ.</t>
+  </si>
+  <si>
+    <t>Nút Đưa Ảnh Xuống Dưới, hoặc gõ ISURVEY_UAV_SEND_BACK.</t>
+  </si>
+  <si>
+    <t>Chèn Ảnh UAV</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_INSERT</t>
+  </si>
+  <si>
+    <t>Giữ chỗ trên Ribbon. Chưa chèn được ảnh UAV.</t>
+  </si>
+  <si>
+    <t>Nút Chèn Ảnh UAV hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Đang làm</t>
+  </si>
+  <si>
+    <t>Nhập DEM &amp; Bề Mặt</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_DEM</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa nhập DEM.</t>
+  </si>
+  <si>
+    <t>Nút Nhập DEM hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Vẽ Đường Đồng Mức</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_CONTOUR</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa vẽ đường đồng mức từ DEM.</t>
+  </si>
+  <si>
+    <t>Nút Vẽ Đường Đồng Mức hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Hệ Tọa Độ UAV</t>
+  </si>
+  <si>
+    <t>ISURVEY_UAV_CRS</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa thiết lập hệ tọa độ UAV.</t>
+  </si>
+  <si>
+    <t>Nút Hệ Tọa Độ UAV hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Nhập Point Cloud</t>
+  </si>
+  <si>
+    <t>ISURVEY_PC_IMPORT</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa nhập đám mây điểm.</t>
+  </si>
+  <si>
+    <t>Nút Nhập Point Cloud hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Lọc Điểm Mặt Đất</t>
+  </si>
+  <si>
+    <t>ISURVEY_PC_FILTER</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa lọc điểm mặt đất.</t>
+  </si>
+  <si>
+    <t>Nút Lọc Điểm Mặt Đất hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Rải Lưới Điểm</t>
+  </si>
+  <si>
+    <t>ISURVEY_PC_GRID</t>
+  </si>
+  <si>
+    <t>Giữ chỗ. Chưa rải lưới điểm.</t>
+  </si>
+  <si>
+    <t>Nút Rải Lưới Điểm hiện báo chưa làm.</t>
+  </si>
+  <si>
+    <t>Khung Bản Đồ</t>
+  </si>
+  <si>
+    <t>ISURVEY_KHUNG</t>
+  </si>
+  <si>
+    <t>KHUNG</t>
+  </si>
+  <si>
+    <t>Khung bản đồ — lưới, Bắc, thước</t>
+  </si>
+  <si>
+    <t>Chèn khung bản đồ TCVN 7285, khổ A0–A4, tỷ lệ 1/200…1/5000, có lưới tọa độ, mũi tên Bắc và thước.</t>
+  </si>
+  <si>
+    <t>KHUNG → chọn khổ, tỷ lệ, kiểu xoay → chỉ tâm khung.</t>
+  </si>
+  <si>
+    <t>1.8.0</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>Khung Bản Vẽ Kỹ Thuật</t>
+  </si>
+  <si>
+    <t>ISURVEY_KHUNG_BV</t>
+  </si>
+  <si>
+    <t>KHUNGBV</t>
+  </si>
+  <si>
+    <t>Khung kỹ thuật — có logo, không lưới</t>
+  </si>
+  <si>
+    <t>Cùng khổ và tỷ lệ với KHUNG, có khung tên và logo, không vẽ lưới.</t>
+  </si>
+  <si>
+    <t>KHUNGBV → chọn khổ, tỷ lệ, kiểu xoay → chỉ tâm.</t>
+  </si>
+  <si>
+    <t>Rải Khung Theo Tuyến</t>
+  </si>
+  <si>
+    <t>ISURVEY_ROUTE_SHEETS</t>
+  </si>
+  <si>
+    <t>RAIKHUNG</t>
+  </si>
+  <si>
+    <t>Rải khung — một layout, nhiều tờ</t>
+  </si>
+  <si>
+    <t>Rải khung in dọc tuyến. Tên cũ DANTRANG không còn.</t>
+  </si>
+  <si>
+    <t>RAIKHUNG → chọn tuyến → khổ, tỷ lệ, hàng cột.</t>
+  </si>
+  <si>
+    <t>1.8.8</t>
+  </si>
+  <si>
+    <t>28/10/2026</t>
+  </si>
+  <si>
+    <t>Rải Khung Mặt Cắt</t>
+  </si>
+  <si>
+    <t>ISURVEY_PROFILE_SHEETS</t>
+  </si>
+  <si>
+    <t>RAIMCD</t>
+  </si>
+  <si>
+    <t>Rải khung mặt cắt dọc</t>
+  </si>
+  <si>
+    <t>Chọn góc dưới-trái hàng cuối. Tỷ lệ trên khung 1/500; 1/5000 hoặc 1/200; 1/2000.</t>
+  </si>
+  <si>
+    <t>RAIMCD → chọn góc → điền khung tên.</t>
+  </si>
+  <si>
+    <t>In Tuyến / Mặt Cắt</t>
+  </si>
+  <si>
+    <t>ISURVEY_ROUTE_PLOT</t>
+  </si>
+  <si>
+    <t>INTUYEN</t>
+  </si>
+  <si>
+    <t>In layout đã rải</t>
+  </si>
+  <si>
+    <t>In layout tuyến hoặc mặt cắt đã có, không dựng trang mới.</t>
+  </si>
+  <si>
+    <t>INTUYEN → gõ 1 khung đang chọn hoặc 2 tất cả.</t>
+  </si>
+  <si>
+    <t>1.8.7</t>
+  </si>
+  <si>
+    <t>Ẩn Logo</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGO</t>
+  </si>
+  <si>
+    <t>ANLOGO</t>
+  </si>
+  <si>
+    <t>Ẩn logo — hỏi 1 hoặc 2</t>
+  </si>
+  <si>
+    <t>Hỏi ẩn logo chủ đầu tư (1) hay đơn vị thiết kế (2).</t>
+  </si>
+  <si>
+    <t>ANLOGO → gõ 1 hoặc 2.</t>
+  </si>
+  <si>
+    <t>1.8.5</t>
+  </si>
+  <si>
+    <t>26/10/2026</t>
+  </si>
+  <si>
+    <t>Ẩn Logo Chủ Đầu Tư</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGO1</t>
+  </si>
+  <si>
+    <t>ANLOGO1</t>
+  </si>
+  <si>
+    <t>Ẩn logo chủ đầu tư</t>
+  </si>
+  <si>
+    <t>Ẩn đúng logo chủ đầu tư.</t>
+  </si>
+  <si>
+    <t>Gõ ANLOGO1.</t>
+  </si>
+  <si>
+    <t>Ẩn Logo Đơn Vị Thiết Kế</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGO2</t>
+  </si>
+  <si>
+    <t>ANLOGO2</t>
+  </si>
+  <si>
+    <t>Ẩn logo đơn vị thiết kế</t>
+  </si>
+  <si>
+    <t>Ẩn đúng logo đơn vị thiết kế.</t>
+  </si>
+  <si>
+    <t>Gõ ANLOGO2.</t>
+  </si>
+  <si>
+    <t>Thay Logo</t>
+  </si>
+  <si>
+    <t>ISURVEY_LOGO_REPLACE</t>
+  </si>
+  <si>
+    <t>THAYLOGO</t>
+  </si>
+  <si>
+    <t>Thay ảnh logo trên khung</t>
+  </si>
+  <si>
+    <t>Đổi file ảnh logo đã gắn trên khung tên.</t>
+  </si>
+  <si>
+    <t>THAYLOGO → chọn logo → chọn ảnh.</t>
+  </si>
+  <si>
+    <t>Co Dãn Chữ Khung Tên</t>
+  </si>
+  <si>
+    <t>ISURVEY_FIT_TITLE</t>
+  </si>
+  <si>
+    <t>CODAN</t>
+  </si>
+  <si>
+    <t>Co chữ khung tên</t>
+  </si>
+  <si>
+    <t>Co chữ ô chủ đầu tư và đại diện về một dòng. Ô tên bản vẽ vẫn xuống dòng.</t>
+  </si>
+  <si>
+    <t>CODAN khi chữ khung tên tràn ô.</t>
+  </si>
+  <si>
+    <t>Tuyến &amp; Cột Điện</t>
+  </si>
+  <si>
+    <t>Đánh Số Góc Tuyến</t>
+  </si>
+  <si>
+    <t>ISURVEY_NUMBER_VERTICES</t>
+  </si>
+  <si>
+    <t>GOC</t>
+  </si>
+  <si>
+    <t>Góc tuyến — số đỉnh tim</t>
+  </si>
+  <si>
+    <t>Đánh số góc tim tuyến, chấm đỏ, chữ né đường.</t>
+  </si>
+  <si>
+    <t>GOC → chọn tim tuyến.</t>
+  </si>
+  <si>
+    <t>Duỗi Thẳng Tuyến</t>
+  </si>
+  <si>
+    <t>ISURVEY_STRIP_MAP</t>
+  </si>
+  <si>
+    <t>DUOITUYEN</t>
+  </si>
+  <si>
+    <t>Duỗi tuyến — ảnh và bảng góc</t>
+  </si>
+  <si>
+    <t>Duỗi ảnh UAV và đối tượng theo tim tuyến, xuất bảng góc.</t>
+  </si>
+  <si>
+    <t>DUOITUYEN → chọn tim → chọn điểm đầu.</t>
+  </si>
+  <si>
+    <t>Đánh Số Thứ Tự</t>
+  </si>
+  <si>
+    <t>Số thứ tự tại điểm chọn</t>
+  </si>
+  <si>
+    <t>Đánh số tại điểm click: tiền tố, hậu tố, bước, chiều cao chữ, vòng tròn. Layer iSurvey_STT.</t>
+  </si>
+  <si>
+    <t>STT → đặt thông số → chọn điểm.</t>
+  </si>
+  <si>
+    <t>29/10/2026</t>
+  </si>
+  <si>
+    <t>Biên tập Địa hình</t>
+  </si>
+  <si>
+    <t>Nhập điểm đo</t>
+  </si>
+  <si>
+    <t>NHAPDIEM</t>
+  </si>
+  <si>
+    <t>Nhập điểm — từ tệp tọa độ</t>
+  </si>
+  <si>
+    <t>Đọc CSV/TXT. Dấu điểm, tên và cao độ mỗi cái một layer, một màu. Xong thì zoom extents.</t>
+  </si>
+  <si>
+    <t>NHAPDIEM → mở tệp → Tạo điểm CAD.</t>
+  </si>
+  <si>
+    <t>Xuất điểm đo</t>
+  </si>
+  <si>
+    <t>XUATDIEM</t>
+  </si>
+  <si>
+    <t>Xuất điểm — ra tệp tọa độ</t>
+  </si>
+  <si>
+    <t>Ghi CSV, cột cách nhau bằng chấm phẩy, thập phân là dấu chấm. Tên xếp từ nhỏ đến lớn, rồi A–Z.</t>
+  </si>
+  <si>
+    <t>XUATDIEM → chọn điểm → Ghi tệp.</t>
+  </si>
+  <si>
+    <t>Trợ lý AI</t>
+  </si>
+  <si>
+    <t>Trợ Lý AI</t>
+  </si>
+  <si>
+    <t>ISURVEY_AI_ASSIST</t>
+  </si>
+  <si>
+    <t>AIA</t>
+  </si>
+  <si>
+    <t>AI assist — chỉ Admin</t>
+  </si>
+  <si>
+    <t>Trợ lý AI khảo sát. Chỉ máy Admin. Đang phát triển.</t>
+  </si>
+  <si>
+    <t>AIA khi đã đăng nhập bằng Gmail Admin.</t>
+  </si>
+  <si>
+    <t>Cấu Hình AI</t>
+  </si>
+  <si>
+    <t>ISURVEY_AI_SETTINGS</t>
+  </si>
+  <si>
+    <t>Thiết lập trợ lý AI. Chỉ Admin. Chưa xong.</t>
+  </si>
+  <si>
+    <t>Nút Cấu Hình AI.</t>
+  </si>
+  <si>
+    <t>Sửa Thông Tin Khung</t>
+  </si>
+  <si>
+    <t>ISURVEY_FRAME_EDIT</t>
+  </si>
+  <si>
+    <t>Sửa chữ và chữ ký trên khung đã chèn. Không cắt lại tuyến. Nhắp đúp khung cũng gọi lệnh này.</t>
+  </si>
+  <si>
+    <t>Nhắp đúp khung, hoặc gõ ISURVEY_FRAME_EDIT rồi chọn khung.</t>
+  </si>
+  <si>
+    <t>UG</t>
+  </si>
+  <si>
+    <t>Update Google — cập nhật ảnh GE</t>
+  </si>
+  <si>
+    <t>AK</t>
+  </si>
+  <si>
+    <t>Ảnh khung — bật hoặc tắt khung ảnh</t>
+  </si>
+  <si>
+    <t>AD</t>
+  </si>
+  <si>
+    <t>Ảnh dưới — đưa ảnh xuống dưới</t>
+  </si>
+  <si>
+    <t>AIC</t>
+  </si>
+  <si>
+    <t>AI cấu hình — chỉ Admin</t>
+  </si>
+  <si>
+    <t>SK</t>
+  </si>
+  <si>
+    <t>Sửa khung — nhắp đúp hoặc gõ SK</t>
+  </si>
+  <si>
+    <t>ND</t>
+  </si>
+  <si>
+    <t>XD</t>
+  </si>
+  <si>
+    <t>AU</t>
+  </si>
+  <si>
+    <t>Ảnh UAV — chèn ảnh, chưa làm</t>
+  </si>
+  <si>
+    <t>DEM</t>
+  </si>
+  <si>
+    <t>DEM — nhập bề mặt, chưa làm</t>
+  </si>
+  <si>
+    <t>DM</t>
+  </si>
+  <si>
+    <t>Đồng mức — chưa vẽ</t>
+  </si>
+  <si>
+    <t>HT</t>
+  </si>
+  <si>
+    <t>Hệ tọa độ UAV — chưa làm</t>
+  </si>
+  <si>
+    <t>NP</t>
+  </si>
+  <si>
+    <t>Nhập point cloud — chưa làm</t>
+  </si>
+  <si>
+    <t>LP</t>
+  </si>
+  <si>
+    <t>Lọc điểm mặt đất — chưa làm</t>
+  </si>
+  <si>
+    <t>RL</t>
+  </si>
+  <si>
+    <t>Rải lưới điểm — chưa làm</t>
+  </si>
+  <si>
+    <t>1.8.10</t>
   </si>
 </sst>
 </file>
@@ -846,22 +1521,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}">
-  <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K48"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
-    <col min="2" max="2" width="12.5546875" customWidth="1"/>
-    <col min="3" max="3" width="24.5546875" customWidth="1"/>
-    <col min="4" max="4" width="22.5546875" customWidth="1"/>
-    <col min="5" max="5" width="10.5546875" customWidth="1"/>
-    <col min="6" max="6" width="36.5546875" customWidth="1"/>
-    <col min="7" max="8" width="48.5546875" customWidth="1"/>
-    <col min="9" max="9" width="10.5546875" customWidth="1"/>
-    <col min="10" max="10" width="14.5546875" style="6" customWidth="1"/>
-    <col min="11" max="11" width="28.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.53125" customWidth="1"/>
+    <col min="2" max="2" width="12.53125" customWidth="1"/>
+    <col min="3" max="3" width="24.53125" customWidth="1"/>
+    <col min="4" max="4" width="22.53125" customWidth="1"/>
+    <col min="5" max="5" width="10.53125" customWidth="1"/>
+    <col min="6" max="6" width="36.53125" customWidth="1"/>
+    <col min="7" max="8" width="48.53125" customWidth="1"/>
+    <col min="9" max="9" width="10.53125" customWidth="1"/>
+    <col min="10" max="10" width="14.53125" style="6" customWidth="1"/>
+    <col min="11" max="11" width="28.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -878,7 +1553,7 @@
         <v>4</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="G1" s="9" t="s">
         <v>5</v>
@@ -896,7 +1571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -910,10 +1585,10 @@
         <v>12</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>13</v>
@@ -925,13 +1600,13 @@
         <v>15</v>
       </c>
       <c r="J2" s="3">
-        <v>46267</v>
+        <v>46062</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -945,10 +1620,10 @@
         <v>18</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>19</v>
@@ -960,13 +1635,13 @@
         <v>15</v>
       </c>
       <c r="J3" s="5">
-        <v>46267</v>
+        <v>46062</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -980,10 +1655,10 @@
         <v>22</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>23</v>
@@ -995,13 +1670,13 @@
         <v>15</v>
       </c>
       <c r="J4" s="3">
-        <v>46267</v>
+        <v>46062</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1015,10 +1690,10 @@
         <v>26</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>59</v>
+        <v>112</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>27</v>
@@ -1030,203 +1705,201 @@
         <v>29</v>
       </c>
       <c r="J5" s="5">
-        <v>46268</v>
+        <v>46090</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="F6" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="H6" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="I6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="J6" s="3">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="4">
         <v>6</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="F7" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="E7" s="8" t="s">
+      <c r="H7" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>84</v>
-      </c>
       <c r="I7" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="J7" s="5">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="F8" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="H8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="I8" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G8" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>92</v>
-      </c>
       <c r="J8" s="3">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="4">
         <v>8</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="J9" s="5">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="J10" s="3">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="4">
         <v>10</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="E11" s="8" t="s">
         <v>107</v>
       </c>
+      <c r="E11" s="8"/>
       <c r="F11" s="8" t="s">
         <v>108</v>
       </c>
@@ -1237,50 +1910,1240 @@
         <v>110</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="J11" s="5">
-        <v>46307</v>
+        <v>46366</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E12" s="7"/>
+        <v>118</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>119</v>
+      </c>
       <c r="F12" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>303</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="J25" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="J26" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>238</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>241</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J27" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>247</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>249</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>266</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="J30" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G31" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="I31" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="J12" s="3">
-        <v>46307</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="J31" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="E32" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K32" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J33" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K33" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="K36" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>284</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="E38" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>291</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="F39" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="I40" s="2"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="I41" s="2"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="I42" s="2"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A43" s="2">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I43" s="2"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="I44" s="2"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="I45" s="2"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A46" s="2">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>338</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>339</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="I46" s="2"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="2"/>
+      <c r="H47" s="2"/>
+      <c r="I47" s="2"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="2"/>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="2"/>
+      <c r="H48" s="2"/>
+      <c r="I48" s="2"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K12" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}"/>
+  <autoFilter ref="A1:K46" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1288,198 +3151,198 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B0ECC91-F81E-481F-BB81-DBB8A841A6BC}">
   <dimension ref="A1:B28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="36.5546875" customWidth="1"/>
-    <col min="2" max="2" width="70.5546875" customWidth="1"/>
+    <col min="1" max="1" width="36.53125" customWidth="1"/>
+    <col min="2" max="2" width="70.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>7</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>8</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>9</v>
       </c>
       <c r="B13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>1</v>
       </c>
       <c r="B15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>3</v>
       </c>
       <c r="B17" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24" s="11" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B25" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="11" t="s">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="B26" t="s">
         <v>62</v>
       </c>
-      <c r="B25" t="s">
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="B27" t="s">
         <v>64</v>
       </c>
-      <c r="B26" t="s">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="B28" t="s">
         <v>66</v>
-      </c>
-      <c r="B27" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" t="s">
-        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sua UPD: dong Civil nhu bam nut dong, hoi luu ban ve chua luu, cai ngay khi da tat.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB198ACD-DB81-4879-BFC7-B44DEC77AD24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8996BCA-69E9-4DAE-9CA0-CDC3A5DB6774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="342">
   <si>
     <t>STT</t>
   </si>
@@ -384,12 +384,6 @@
     <t>Export Google / Export KML — xuất KML/KMZ</t>
   </si>
   <si>
-    <t>Kiểm tra bản mới. Có bản thì tải và cài sau khi thoát Civil.</t>
-  </si>
-  <si>
-    <t>UPD hoặc nút Kiểm Tra Cập Nhật → Cập nhật ngay / Đóng.</t>
-  </si>
-  <si>
     <t>1.8.6</t>
   </si>
   <si>
@@ -1066,6 +1060,15 @@
   </si>
   <si>
     <t>1.8.10</t>
+  </si>
+  <si>
+    <t>Tải gói và giải nén. Rồi đóng Civil như bấm nút đóng. Bản vẽ chưa lưu thì hỏi lưu. Tắt xong thì cài ngay.</t>
+  </si>
+  <si>
+    <t>UPD hoặc nút Kiểm Tra Cập Nhật. Bấm Cập nhật ngay. Nếu bản vẽ chưa lưu thì chọn lưu hoặc không lưu.</t>
+  </si>
+  <si>
+    <t>1.8.11</t>
   </si>
 </sst>
 </file>
@@ -1927,28 +1930,28 @@
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="E12" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="G12" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="H12" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="J12" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>16</v>
@@ -1962,28 +1965,28 @@
         <v>10</v>
       </c>
       <c r="C13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>313</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>314</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>128</v>
-      </c>
       <c r="I13" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>16</v>
@@ -1997,28 +2000,28 @@
         <v>10</v>
       </c>
       <c r="C14" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="F14" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="G14" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="H14" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="J14" s="3" t="s">
         <v>142</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>144</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>16</v>
@@ -2032,28 +2035,28 @@
         <v>10</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="F15" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="G15" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="H15" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="G15" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="I15" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>16</v>
@@ -2067,28 +2070,28 @@
         <v>10</v>
       </c>
       <c r="C16" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="F16" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="G16" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="H16" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="G16" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>156</v>
-      </c>
       <c r="I16" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>16</v>
@@ -2099,31 +2102,31 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="E17" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="F17" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="G17" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="H17" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="J17" s="3" t="s">
         <v>163</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>165</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>16</v>
@@ -2134,31 +2137,31 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C18" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="H18" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E18" s="7" t="s">
-        <v>316</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>317</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>169</v>
-      </c>
       <c r="I18" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>16</v>
@@ -2169,31 +2172,31 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E19" s="7" t="s">
-        <v>318</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="I19" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>16</v>
@@ -2204,31 +2207,31 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="G20" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="H20" s="2" t="s">
         <v>274</v>
       </c>
-      <c r="G20" s="2" t="s">
-        <v>275</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>276</v>
-      </c>
       <c r="I20" s="2" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>16</v>
@@ -2242,28 +2245,28 @@
         <v>67</v>
       </c>
       <c r="C21" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="D21" s="2" t="s">
+      <c r="F21" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="G21" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="H21" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="I21" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="J21" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="I21" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="J21" s="3" t="s">
-        <v>210</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>16</v>
@@ -2277,28 +2280,28 @@
         <v>67</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="E22" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="F22" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="G22" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="H22" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="G22" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>216</v>
-      </c>
       <c r="I22" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>16</v>
@@ -2309,31 +2312,31 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="E23" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="F23" s="7" t="s">
         <v>278</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="G23" s="2" t="s">
         <v>279</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="H23" s="2" t="s">
         <v>280</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>281</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>282</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>16</v>
@@ -2344,34 +2347,34 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>299</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="E24" s="7" t="s">
         <v>300</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="7" t="s">
         <v>301</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="G24" s="2" t="s">
         <v>302</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="H24" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>305</v>
-      </c>
       <c r="I24" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.45">
@@ -2379,34 +2382,34 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C25" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>318</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>319</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="D25" s="2" t="s">
+      <c r="H25" s="2" t="s">
         <v>307</v>
       </c>
-      <c r="E25" s="7" t="s">
-        <v>320</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>309</v>
-      </c>
       <c r="I25" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
@@ -2417,28 +2420,28 @@
         <v>10</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="F26" s="7" t="s">
         <v>130</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="G26" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="H26" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="I26" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="H26" s="2" t="s">
+      <c r="J26" s="3" t="s">
         <v>134</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>136</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>16</v>
@@ -2452,28 +2455,28 @@
         <v>67</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>236</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>238</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="F27" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="G27" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="H27" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="J27" s="3" t="s">
         <v>243</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>245</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>16</v>
@@ -2487,28 +2490,28 @@
         <v>67</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E28" s="7" t="s">
         <v>246</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="F28" s="7" t="s">
         <v>247</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="G28" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="H28" s="2" t="s">
         <v>249</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>251</v>
-      </c>
       <c r="I28" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>16</v>
@@ -2522,28 +2525,28 @@
         <v>67</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>252</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="G29" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="H29" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>256</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>257</v>
-      </c>
       <c r="I29" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>16</v>
@@ -2557,28 +2560,28 @@
         <v>67</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="F30" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="G30" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="H30" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>268</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>269</v>
-      </c>
       <c r="I30" s="2" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>16</v>
@@ -2604,16 +2607,16 @@
         <v>93</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>113</v>
+        <v>339</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>114</v>
+        <v>340</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>115</v>
+        <v>341</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>116</v>
+        <v>285</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>16</v>
@@ -2627,28 +2630,28 @@
         <v>67</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="E32" s="7" t="s">
         <v>258</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="7" t="s">
         <v>259</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="G32" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="H32" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="G32" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>263</v>
-      </c>
       <c r="I32" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K32" s="2" t="s">
         <v>16</v>
@@ -2662,28 +2665,28 @@
         <v>67</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>321</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>310</v>
       </c>
-      <c r="D33" s="2" t="s">
+      <c r="H33" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="E33" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="F33" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>313</v>
-      </c>
       <c r="I33" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>16</v>
@@ -2697,28 +2700,28 @@
         <v>67</v>
       </c>
       <c r="C34" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="E34" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="D34" s="2" t="s">
+      <c r="F34" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="G34" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="H34" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="I34" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="H34" s="2" t="s">
-        <v>236</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>237</v>
-      </c>
       <c r="J34" s="3" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>16</v>
@@ -2732,28 +2735,28 @@
         <v>67</v>
       </c>
       <c r="C35" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="E35" s="7" t="s">
         <v>217</v>
       </c>
-      <c r="D35" s="2" t="s">
+      <c r="F35" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="G35" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="H35" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="I35" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="H35" s="2" t="s">
+      <c r="J35" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>224</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>16</v>
@@ -2767,28 +2770,28 @@
         <v>67</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="D36" s="2" t="s">
+      <c r="F36" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E36" s="7" t="s">
+      <c r="G36" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="F36" s="7" t="s">
+      <c r="H36" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="I36" s="2" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>16</v>
@@ -2799,10 +2802,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>0</v>
@@ -2811,19 +2814,19 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="I37" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>285</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>286</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>16</v>
@@ -2834,31 +2837,31 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="E38" s="7" t="s">
+        <v>322</v>
+      </c>
+      <c r="F38" s="7" t="s">
         <v>289</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="F38" s="7" t="s">
+      <c r="H38" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>292</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>293</v>
-      </c>
       <c r="I38" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>16</v>
@@ -2869,31 +2872,31 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>323</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>294</v>
       </c>
-      <c r="D39" s="2" t="s">
+      <c r="G39" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="E39" s="7" t="s">
-        <v>325</v>
-      </c>
-      <c r="F39" s="7" t="s">
+      <c r="H39" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="G39" s="2" t="s">
-        <v>297</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="I39" s="2" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>16</v>
@@ -2904,30 +2907,30 @@
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C40" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="F40" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="G40" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="H40" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>326</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>327</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H40" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="3"/>
       <c r="K40" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.45">
@@ -2935,30 +2938,30 @@
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C41" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>326</v>
+      </c>
+      <c r="F41" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="G41" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="D41" s="2" t="s">
+      <c r="H41" s="2" t="s">
         <v>180</v>
-      </c>
-      <c r="E41" s="7" t="s">
-        <v>328</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>329</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="H41" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="I41" s="2"/>
       <c r="J41" s="3"/>
       <c r="K41" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.45">
@@ -2966,30 +2969,30 @@
         <v>41</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="D42" s="2" t="s">
+      <c r="H42" s="2" t="s">
         <v>184</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>185</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>186</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="3"/>
       <c r="K42" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.45">
@@ -2997,30 +3000,30 @@
         <v>42</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C43" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="G43" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="D43" s="2" t="s">
+      <c r="H43" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>333</v>
-      </c>
-      <c r="G43" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="H43" s="2" t="s">
-        <v>190</v>
       </c>
       <c r="I43" s="2"/>
       <c r="J43" s="3"/>
       <c r="K43" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.45">
@@ -3028,30 +3031,30 @@
         <v>43</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C44" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="F44" s="7" t="s">
+        <v>333</v>
+      </c>
+      <c r="G44" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="D44" s="2" t="s">
+      <c r="H44" s="2" t="s">
         <v>192</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>334</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="G44" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="H44" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="I44" s="2"/>
       <c r="J44" s="3"/>
       <c r="K44" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.45">
@@ -3059,30 +3062,30 @@
         <v>44</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E45" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="F45" s="7" t="s">
+        <v>335</v>
+      </c>
+      <c r="G45" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="D45" s="2" t="s">
+      <c r="H45" s="2" t="s">
         <v>196</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>336</v>
-      </c>
-      <c r="F45" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="G45" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="H45" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="I45" s="2"/>
       <c r="J45" s="3"/>
       <c r="K45" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.45">
@@ -3090,30 +3093,30 @@
         <v>45</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C46" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="F46" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="G46" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="D46" s="2" t="s">
+      <c r="H46" s="2" t="s">
         <v>200</v>
-      </c>
-      <c r="E46" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="F46" s="7" t="s">
-        <v>339</v>
-      </c>
-      <c r="G46" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="H46" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="3"/>
       <c r="K46" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Sua UPD 1.8.13: dong Civil ngay sau khi giai nen, chon khong luu van cai.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8996BCA-69E9-4DAE-9CA0-CDC3A5DB6774}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF9D6B8-1E0A-4DE8-BD2A-45A0B06DBB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
@@ -1068,7 +1068,7 @@
     <t>UPD hoặc nút Kiểm Tra Cập Nhật. Bấm Cập nhật ngay. Nếu bản vẽ chưa lưu thì chọn lưu hoặc không lưu.</t>
   </si>
   <si>
-    <t>1.8.11</t>
+    <t>1.8.13</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Phat hanh 1.8.14: HD mo huong dan web, xuat diem tu chu va block, in PDF co moc do va nut mo thu muc.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF9D6B8-1E0A-4DE8-BD2A-45A0B06DBB12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08AA9096-BB80-4C90-9AE2-7FA59A864CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Mau chuan" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Danh sach lenh'!$A$1:$K$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="350">
   <si>
     <t>STT</t>
   </si>
@@ -744,15 +744,9 @@
     <t>In layout đã rải</t>
   </si>
   <si>
-    <t>In layout tuyến hoặc mặt cắt đã có, không dựng trang mới.</t>
-  </si>
-  <si>
     <t>INTUYEN → gõ 1 khung đang chọn hoặc 2 tất cả.</t>
   </si>
   <si>
-    <t>1.8.7</t>
-  </si>
-  <si>
     <t>Ẩn Logo</t>
   </si>
   <si>
@@ -930,12 +924,6 @@
     <t>Xuất điểm — ra tệp tọa độ</t>
   </si>
   <si>
-    <t>Ghi CSV, cột cách nhau bằng chấm phẩy, thập phân là dấu chấm. Tên xếp từ nhỏ đến lớn, rồi A–Z.</t>
-  </si>
-  <si>
-    <t>XUATDIEM → chọn điểm → Ghi tệp.</t>
-  </si>
-  <si>
     <t>Trợ lý AI</t>
   </si>
   <si>
@@ -975,12 +963,6 @@
     <t>ISURVEY_FRAME_EDIT</t>
   </si>
   <si>
-    <t>Sửa chữ và chữ ký trên khung đã chèn. Không cắt lại tuyến. Nhắp đúp khung cũng gọi lệnh này.</t>
-  </si>
-  <si>
-    <t>Nhắp đúp khung, hoặc gõ ISURVEY_FRAME_EDIT rồi chọn khung.</t>
-  </si>
-  <si>
     <t>UG</t>
   </si>
   <si>
@@ -1069,6 +1051,48 @@
   </si>
   <si>
     <t>1.8.13</t>
+  </si>
+  <si>
+    <t>Sửa chữ và chữ ký DWG trên khung đã chèn. Mộc đỏ (PNG) chỉ đóng khi xuất PDF, không nằm trong bản vẽ. Nhắp đúp khung cũng gọi lệnh này.</t>
+  </si>
+  <si>
+    <t>Nhắp đúp khung hoặc gõ SK. Dòng họ tên: Đổi chữ ký hoặc Xóa. Chân hộp thoại: chọn ảnh PNG nếu muốn đóng dấu lúc xuất PDF.</t>
+  </si>
+  <si>
+    <t>30/10/2026</t>
+  </si>
+  <si>
+    <t>In layout tuyến hoặc mặt cắt đã có, không dựng trang mới. In xong có nút Mở thư mục.</t>
+  </si>
+  <si>
+    <t>Chọn Point, Block, Text hoặc MText rồi ghi CSV hoặc TXT. CSV dùng dấu phân cách của máy. TXT dùng tab. Thập phân là dấu chấm. Tên xếp từ nhỏ đến lớn.</t>
+  </si>
+  <si>
+    <t>XUATDIEM. Bấm Chọn số liệu trên bản vẽ, rồi Xuất tệp. Chữ đọc được thành số thì thành cao độ. Nút Xuất tệp chỉ bật khi đã chọn điểm.</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>Hướng dẫn</t>
+  </si>
+  <si>
+    <t>ISURVEY_HDSD</t>
+  </si>
+  <si>
+    <t>HD</t>
+  </si>
+  <si>
+    <t>HDSD — mở hướng dẫn trên web</t>
+  </si>
+  <si>
+    <t>Mở trang hướng dẫn iSurvey trên trình duyệt. Không cần đăng nhập.</t>
+  </si>
+  <si>
+    <t>HD hoặc nút Hướng dẫn trong Tài khoản và Hệ thống.</t>
+  </si>
+  <si>
+    <t>1.8.14</t>
   </si>
 </sst>
 </file>
@@ -1161,7 +1185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1190,6 +1214,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1971,10 +2001,10 @@
         <v>124</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>125</v>
@@ -2146,10 +2176,10 @@
         <v>165</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>166</v>
@@ -2181,10 +2211,10 @@
         <v>169</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>170</v>
@@ -2207,25 +2237,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="7" t="s">
         <v>270</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="G20" s="2" t="s">
         <v>271</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="H20" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>273</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>274</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>162</v>
@@ -2312,25 +2342,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C23" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="E23" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="F23" s="7" t="s">
         <v>276</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="G23" s="2" t="s">
         <v>277</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="H23" s="2" t="s">
         <v>278</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>207</v>
@@ -2347,25 +2377,25 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="F24" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="G24" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="D24" s="2" t="s">
+      <c r="H24" s="2" t="s">
         <v>299</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>300</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>301</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>303</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>207</v>
@@ -2382,25 +2412,25 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>207</v>
@@ -2455,28 +2485,28 @@
         <v>67</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="E27" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="D27" s="2" t="s">
+      <c r="F27" s="7" t="s">
         <v>237</v>
       </c>
-      <c r="E27" s="7" t="s">
+      <c r="G27" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="H27" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="J27" s="3" t="s">
         <v>241</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>242</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>16</v>
@@ -2490,28 +2520,28 @@
         <v>67</v>
       </c>
       <c r="C28" s="2" t="s">
+        <v>242</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="E28" s="7" t="s">
         <v>244</v>
       </c>
-      <c r="D28" s="2" t="s">
+      <c r="F28" s="7" t="s">
         <v>245</v>
       </c>
-      <c r="E28" s="7" t="s">
+      <c r="G28" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="H28" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>249</v>
-      </c>
       <c r="I28" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>16</v>
@@ -2525,28 +2555,28 @@
         <v>67</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="E29" s="7" t="s">
         <v>250</v>
       </c>
-      <c r="D29" s="2" t="s">
+      <c r="F29" s="7" t="s">
         <v>251</v>
       </c>
-      <c r="E29" s="7" t="s">
+      <c r="G29" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="H29" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>254</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>255</v>
-      </c>
       <c r="I29" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>16</v>
@@ -2560,28 +2590,28 @@
         <v>67</v>
       </c>
       <c r="C30" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="D30" s="2" t="s">
+      <c r="F30" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="E30" s="7" t="s">
+      <c r="G30" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="H30" s="2" t="s">
         <v>265</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>267</v>
-      </c>
       <c r="I30" s="2" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>16</v>
@@ -2607,16 +2637,16 @@
         <v>93</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>16</v>
@@ -2630,22 +2660,22 @@
         <v>67</v>
       </c>
       <c r="C32" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="E32" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="E32" s="7" t="s">
+      <c r="G32" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="H32" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>260</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>261</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>113</v>
@@ -2657,7 +2687,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A33" s="2">
         <v>32</v>
       </c>
@@ -2665,28 +2695,28 @@
         <v>67</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>310</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="J33" s="3" t="s">
-        <v>114</v>
+        <v>315</v>
+      </c>
+      <c r="G33" s="12" t="s">
+        <v>336</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>337</v>
+      </c>
+      <c r="I33" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>338</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>16</v>
@@ -2711,17 +2741,17 @@
       <c r="F34" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="12" t="s">
+        <v>339</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="H34" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="I34" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>114</v>
+      <c r="I34" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>338</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>16</v>
@@ -2802,10 +2832,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>0</v>
@@ -2814,19 +2844,19 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>281</v>
+      </c>
+      <c r="H37" s="2" t="s">
         <v>282</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="I37" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>283</v>
-      </c>
-      <c r="H37" s="2" t="s">
-        <v>284</v>
-      </c>
-      <c r="I37" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>16</v>
@@ -2837,66 +2867,66 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>285</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>286</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="E38" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="F38" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="D38" s="2" t="s">
+      <c r="G38" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>322</v>
-      </c>
-      <c r="F38" s="7" t="s">
+      <c r="H38" s="2" t="s">
         <v>289</v>
       </c>
-      <c r="G38" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>291</v>
-      </c>
       <c r="I38" s="2" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>292</v>
       </c>
-      <c r="D39" s="2" t="s">
-        <v>293</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>294</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="H39" s="2" t="s">
-        <v>296</v>
-      </c>
-      <c r="I39" s="2" t="s">
+      <c r="G39" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="I39" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="J39" s="12" t="s">
         <v>338</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>285</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>16</v>
@@ -2916,10 +2946,10 @@
         <v>173</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>174</v>
@@ -2947,10 +2977,10 @@
         <v>178</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>179</v>
@@ -2978,10 +3008,10 @@
         <v>182</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>183</v>
@@ -3009,10 +3039,10 @@
         <v>186</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>187</v>
@@ -3040,10 +3070,10 @@
         <v>190</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>191</v>
@@ -3071,10 +3101,10 @@
         <v>194</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>195</v>
@@ -3102,10 +3132,10 @@
         <v>198</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>199</v>
@@ -3119,18 +3149,40 @@
         <v>176</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="3"/>
-      <c r="K47" s="2"/>
+    <row r="47" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+      <c r="A47" s="12" t="s">
+        <v>342</v>
+      </c>
+      <c r="B47" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>345</v>
+      </c>
+      <c r="F47" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="G47" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>348</v>
+      </c>
+      <c r="I47" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="J47" s="12" t="s">
+        <v>338</v>
+      </c>
+      <c r="K47" s="12" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A48" s="2"/>
@@ -3146,7 +3198,7 @@
       <c r="K48" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K46" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}"/>
+  <autoFilter ref="A1:K48" xr:uid="{90AF593E-BDB0-41BC-9C56-B6BF739C3D56}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Giu 1.8.14: rai khung chi dung layout, INTUYEN moi chon kieu in va chu ky theo chuc danh.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="d:\AIProject\isurvey\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08AA9096-BB80-4C90-9AE2-7FA59A864CDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC058B1D-57F9-424F-B22F-932B3F711684}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="1" xr2:uid="{4D0B335C-460A-4570-B0C9-3B46DE2B1793}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="348">
   <si>
     <t>STT</t>
   </si>
@@ -702,18 +702,6 @@
     <t>Rải khung — một layout, nhiều tờ</t>
   </si>
   <si>
-    <t>Rải khung in dọc tuyến. Tên cũ DANTRANG không còn.</t>
-  </si>
-  <si>
-    <t>RAIKHUNG → chọn tuyến → khổ, tỷ lệ, hàng cột.</t>
-  </si>
-  <si>
-    <t>1.8.8</t>
-  </si>
-  <si>
-    <t>28/10/2026</t>
-  </si>
-  <si>
     <t>Rải Khung Mặt Cắt</t>
   </si>
   <si>
@@ -726,12 +714,6 @@
     <t>Rải khung mặt cắt dọc</t>
   </si>
   <si>
-    <t>Chọn góc dưới-trái hàng cuối. Tỷ lệ trên khung 1/500; 1/5000 hoặc 1/200; 1/2000.</t>
-  </si>
-  <si>
-    <t>RAIMCD → chọn góc → điền khung tên.</t>
-  </si>
-  <si>
     <t>In Tuyến / Mặt Cắt</t>
   </si>
   <si>
@@ -744,9 +726,6 @@
     <t>In layout đã rải</t>
   </si>
   <si>
-    <t>INTUYEN → gõ 1 khung đang chọn hoặc 2 tất cả.</t>
-  </si>
-  <si>
     <t>Ẩn Logo</t>
   </si>
   <si>
@@ -1062,9 +1041,6 @@
     <t>30/10/2026</t>
   </si>
   <si>
-    <t>In layout tuyến hoặc mặt cắt đã có, không dựng trang mới. In xong có nút Mở thư mục.</t>
-  </si>
-  <si>
     <t>Chọn Point, Block, Text hoặc MText rồi ghi CSV hoặc TXT. CSV dùng dấu phân cách của máy. TXT dùng tab. Thập phân là dấu chấm. Tên xếp từ nhỏ đến lớn.</t>
   </si>
   <si>
@@ -1093,6 +1069,24 @@
   </si>
   <si>
     <t>1.8.14</t>
+  </si>
+  <si>
+    <t>In layout đã rải. Hỏi in màu hoặc đen trắng, chèn chữ ký và đóng mộc. Chữ ký và mộc chỉ trên PDF. In xong có nút Mở thư mục.</t>
+  </si>
+  <si>
+    <t>Rải khung in dọc tuyến, chỉ dựng layout. Không in PDF ở bước này. Tên cũ DANTRANG không còn.</t>
+  </si>
+  <si>
+    <t>RAIKHUNG → chọn tuyến → khổ, tỷ lệ, hàng cột. In sau bằng INTUYEN.</t>
+  </si>
+  <si>
+    <t>Rải khung mặt cắt đã vẽ, chỉ dựng layout. Không in PDF ở bước này.</t>
+  </si>
+  <si>
+    <t>RAIMCD → chọn góc → điền khung tên. In sau bằng INTUYEN.</t>
+  </si>
+  <si>
+    <t>INTUYEN → chọn kiểu in, chữ ký theo chức danh trên khung, mộc → gõ 1 hoặc 2 → chọn file PDF.</t>
   </si>
 </sst>
 </file>
@@ -2001,10 +1995,10 @@
         <v>124</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>125</v>
@@ -2176,10 +2170,10 @@
         <v>165</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>308</v>
+        <v>301</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>309</v>
+        <v>302</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>166</v>
@@ -2211,10 +2205,10 @@
         <v>169</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>311</v>
+        <v>304</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>170</v>
@@ -2237,25 +2231,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>162</v>
@@ -2342,25 +2336,25 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>266</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>273</v>
-      </c>
       <c r="D23" s="2" t="s">
-        <v>274</v>
+        <v>267</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>207</v>
@@ -2377,25 +2371,25 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>207</v>
@@ -2412,25 +2406,25 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>300</v>
-      </c>
       <c r="D25" s="2" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>312</v>
+        <v>305</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>313</v>
+        <v>306</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>207</v>
@@ -2485,28 +2479,28 @@
         <v>67</v>
       </c>
       <c r="C27" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="J27" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>235</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>239</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>241</v>
       </c>
       <c r="K27" s="2" t="s">
         <v>16</v>
@@ -2520,28 +2514,28 @@
         <v>67</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>16</v>
@@ -2555,28 +2549,28 @@
         <v>67</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>16</v>
@@ -2590,28 +2584,28 @@
         <v>67</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="K30" s="2" t="s">
         <v>16</v>
@@ -2637,16 +2631,16 @@
         <v>93</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>334</v>
+        <v>327</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>335</v>
+        <v>328</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="K31" s="2" t="s">
         <v>16</v>
@@ -2660,22 +2654,22 @@
         <v>67</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>113</v>
@@ -2695,34 +2689,34 @@
         <v>67</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>314</v>
+        <v>307</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="G33" s="12" t="s">
-        <v>336</v>
+        <v>329</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>337</v>
+        <v>330</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="J33" s="12" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="K33" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A34" s="2">
         <v>33</v>
       </c>
@@ -2730,28 +2724,28 @@
         <v>67</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="G34" s="12" t="s">
-        <v>339</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>233</v>
+        <v>342</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>347</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="J34" s="12" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="K34" s="2" t="s">
         <v>16</v>
@@ -2776,17 +2770,17 @@
       <c r="F35" s="7" t="s">
         <v>218</v>
       </c>
-      <c r="G35" s="2" t="s">
-        <v>219</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>222</v>
+      <c r="G35" s="12" t="s">
+        <v>343</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>344</v>
+      </c>
+      <c r="I35" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>331</v>
       </c>
       <c r="K35" s="2" t="s">
         <v>16</v>
@@ -2800,28 +2794,28 @@
         <v>67</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="G36" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>221</v>
-      </c>
-      <c r="J36" s="3" t="s">
         <v>222</v>
+      </c>
+      <c r="G36" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>346</v>
+      </c>
+      <c r="I36" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="J36" s="12" t="s">
+        <v>331</v>
       </c>
       <c r="K36" s="2" t="s">
         <v>16</v>
@@ -2832,10 +2826,10 @@
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="D37" s="2" t="s">
         <v>0</v>
@@ -2844,19 +2838,19 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="K37" s="2" t="s">
         <v>16</v>
@@ -2867,31 +2861,31 @@
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>316</v>
+        <v>309</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>332</v>
+        <v>325</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="K38" s="2" t="s">
         <v>16</v>
@@ -2902,31 +2896,31 @@
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>284</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>291</v>
-      </c>
       <c r="E39" s="7" t="s">
-        <v>317</v>
+        <v>310</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="G39" s="12" t="s">
-        <v>340</v>
+        <v>332</v>
       </c>
       <c r="H39" s="12" t="s">
+        <v>333</v>
+      </c>
+      <c r="I39" s="12" t="s">
         <v>341</v>
       </c>
-      <c r="I39" s="12" t="s">
-        <v>349</v>
-      </c>
       <c r="J39" s="12" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="K39" s="2" t="s">
         <v>16</v>
@@ -2946,10 +2940,10 @@
         <v>173</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>318</v>
+        <v>311</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
       <c r="G40" s="2" t="s">
         <v>174</v>
@@ -2977,10 +2971,10 @@
         <v>178</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>320</v>
+        <v>313</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>321</v>
+        <v>314</v>
       </c>
       <c r="G41" s="2" t="s">
         <v>179</v>
@@ -3008,10 +3002,10 @@
         <v>182</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>322</v>
+        <v>315</v>
       </c>
       <c r="F42" s="7" t="s">
-        <v>323</v>
+        <v>316</v>
       </c>
       <c r="G42" s="2" t="s">
         <v>183</v>
@@ -3039,10 +3033,10 @@
         <v>186</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>324</v>
+        <v>317</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>325</v>
+        <v>318</v>
       </c>
       <c r="G43" s="2" t="s">
         <v>187</v>
@@ -3070,10 +3064,10 @@
         <v>190</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>326</v>
+        <v>319</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>327</v>
+        <v>320</v>
       </c>
       <c r="G44" s="2" t="s">
         <v>191</v>
@@ -3101,10 +3095,10 @@
         <v>194</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>328</v>
+        <v>321</v>
       </c>
       <c r="F45" s="7" t="s">
-        <v>329</v>
+        <v>322</v>
       </c>
       <c r="G45" s="2" t="s">
         <v>195</v>
@@ -3132,10 +3126,10 @@
         <v>198</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>330</v>
+        <v>323</v>
       </c>
       <c r="F46" s="7" t="s">
-        <v>331</v>
+        <v>324</v>
       </c>
       <c r="G46" s="2" t="s">
         <v>199</v>
@@ -3151,34 +3145,34 @@
     </row>
     <row r="47" spans="1:11" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A47" s="12" t="s">
-        <v>342</v>
+        <v>334</v>
       </c>
       <c r="B47" s="12" t="s">
         <v>82</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>343</v>
+        <v>335</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>344</v>
+        <v>336</v>
       </c>
       <c r="E47" s="13" t="s">
-        <v>345</v>
+        <v>337</v>
       </c>
       <c r="F47" s="13" t="s">
-        <v>346</v>
+        <v>338</v>
       </c>
       <c r="G47" s="12" t="s">
-        <v>347</v>
+        <v>339</v>
       </c>
       <c r="H47" s="12" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="I47" s="12" t="s">
-        <v>349</v>
+        <v>341</v>
       </c>
       <c r="J47" s="12" t="s">
-        <v>338</v>
+        <v>331</v>
       </c>
       <c r="K47" s="12" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Ghi vỏ BANGIS 1.8.15: bảng nền xám, icon từng mục, chưa phát hành.
Cây chưa đọc bản vẽ. RAIMCD vẫn chỉ rải khung.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="5.53125" customWidth="1" min="1" max="1"/>
@@ -1396,11 +1396,13 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>1.8.14</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>46325</v>
+          <t>1.8.15</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
@@ -2384,7 +2386,7 @@
       </c>
       <c r="I34" s="12" t="inlineStr">
         <is>
-          <t>1.8.14</t>
+          <t>1.8.15</t>
         </is>
       </c>
       <c r="J34" s="12" t="inlineStr">
@@ -2439,7 +2441,7 @@
       </c>
       <c r="I35" s="12" t="inlineStr">
         <is>
-          <t>1.8.14</t>
+          <t>1.8.15</t>
         </is>
       </c>
       <c r="J35" s="12" t="inlineStr">
@@ -2494,7 +2496,7 @@
       </c>
       <c r="I36" s="12" t="inlineStr">
         <is>
-          <t>1.8.14</t>
+          <t>1.8.15</t>
         </is>
       </c>
       <c r="J36" s="12" t="inlineStr">
@@ -3100,7 +3102,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>1.8.14</t>
+          <t>1.8.15</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
@@ -3109,6 +3111,61 @@
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
+        <is>
+          <t>Đang làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Dữ liệu</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bảng dữ liệu</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ISURVEY_PALETTE</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>BANGIS</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Bảng dữ liệu — vỏ palette</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Mở hoặc đóng bảng neo trái. Nền xám, mỗi mục có icon. Bốn tab Khảo sát, Khung in, UAV, Bản đồ. Cây chưa đọc bản vẽ.</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>BANGIS hoặc nút Bảng dữ liệu. Cần đăng nhập.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>1.8.15</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>30/10/2026</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>Đang làm</t>
         </is>

</xml_diff>

<commit_message>
Ghi pha 1 mô hình 1.8.16: lưới không cạnh dài, đứt gãy là cạnh bắt buộc, chưa phát hành.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_lenh_iSurvey.xlsx
+++ b/docs/Danh_sach_lenh_iSurvey.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="5.53125" customWidth="1" min="1" max="1"/>
@@ -2596,22 +2596,22 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Đọc CSV/TXT. Dấu điểm, tên và cao độ mỗi cái một layer, một màu. Xong thì zoom extents.</t>
+          <t>Bảng giữ X Bắc và Y Đông. Khi vẽ, CAD nhận Đông trên trục X và Bắc trên trục Y. Có cao chữ, kiểu điểm và cỡ điểm theo phần trăm.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>NHAPDIEM → mở tệp → Tạo điểm CAD.</t>
+          <t>NHAPDIEM → mở tệp → chọn kiểu điểm → Nhập điểm.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>1.8.10</t>
+          <t>1.8.16</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>29/10/2026</t>
+          <t>31/10/2026</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Mở hoặc đóng bảng neo trái. Nền xám, mỗi mục có icon. Bốn tab Khảo sát, Khung in, UAV, Bản đồ. Cây chưa đọc bản vẽ.</t>
+          <t>Mở hoặc đóng bảng neo trái. Nền xám, mỗi mục có icon. Bốn tab Khảo sát, Khung in, UAV, Bản đồ. Cây hiện mô hình địa hình đã lưu trong bản vẽ.</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3157,17 +3157,292 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>1.8.15</t>
+          <t>1.8.16</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>30/10/2026</t>
+          <t>31/10/2026</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Đang làm</t>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Biên tập Địa hình</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Tạo mô hình</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ISURVEY_TERRAIN_NEW</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>TAOMOHINH</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Tạo mô hình — vỏ đặt tên</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Tạo mô hình địa hình trong bản vẽ: tên và lớp lưới. Không có cạnh dài nhất. Chưa có tam giác.</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>TAOMOHINH → nhập tên và lớp → Tạo mô hình. Rồi thêm dữ liệu và xây dựng.</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>1.8.16</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Biên tập Địa hình</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Thêm vào mô hình</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ISURVEY_TERRAIN_ADD</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>THEMMOHINH</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Thêm điểm, đứt gãy, đồng mức hoặc bao</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Gắn điểm đo, đường đứt gãy, đường đồng mức hoặc đường bao kín vào mô hình đang chọn. Đứt gãy và đồng mức sẽ thành cạnh bắt buộc khi xây dựng.</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>THEMMOHINH → chọn Điểm, Đứt gãy, Đồng mức hoặc Bao → chọn đối tượng trên bản vẽ.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1.8.16</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Biên tập Địa hình</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Xây dựng mô hình</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ISURVEY_TERRAIN_BUILD</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>XAYMOHINH</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Xây dựng lưới tam giác</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Dựng lưới từ điểm đã gắn. Đứt gãy và đồng mức là cạnh bắt buộc. Có đường bao thì chỉ giữ tam giác trong bao. Không có bao thì lưới là bao lồi.</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>XAYMOHINH. Nên có đường bao trước. Lưới nằm trên lớp của mô hình.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>1.8.16</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Biên tập Địa hình</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Ẩn / Hiện Lưới TIN</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ISURVEY_TERRAIN_TOGGLE</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ANTIN</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Ẩn hoặc hiện lưới</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Ẩn hoặc hiện các mặt tam giác của mô hình. Tra cao độ vẫn dùng lưới đã xây.</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>ANTIN. Trên bảng thì chuột phải tên mô hình.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>1.8.16</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Biên tập Địa hình</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Tra cao độ</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ISURVEY_TERRAIN_Z</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TRACAOD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Tra cao độ trên lưới</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Lấy cao độ nội suy tại một điểm nằm trong lưới đã xây dựng.</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>TRACAOD → chọn một điểm trên bản vẽ.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>1.8.16</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>31/10/2026</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>